<commit_message>
docs: actualizar story points finales y asignación equilibrada de HUs (#46)
- Se actualizaron los story points del Excel con los números finales acordados por el equipo.
- Se eliminaron las justificaciones de puntaje para mantener el documento más limpio. Esto no afectará debido a que fue un agregado no solicitado en algún momento.
- Se repartieron las 22 HUs entre los 5 miembros del grupo dejando la carga balanceada (puntos y cantidad).
- Se asignó la columna "Asignado a" en el Excel usando los nombres exactos para que calce con las fórmulas de excel, y también se reflejó en el README del backend.
- Respetamos las dependencias entre HUs (ACD, MAT, IPN).
- Se actualizaron los story points y los assignees de todos los issues en GitHub (incluyendo los sub-issues de docs y pruebas).
</commit_message>
<xml_diff>
--- a/Documentacion/1. Story Points y Asignacion de Responsabilidades.xlsx
+++ b/Documentacion/1. Story Points y Asignacion de Responsabilidades.xlsx
@@ -32,6 +32,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={04CB6911-E216-5FFA-A00E-331AF1FB8FD4}</author>
+    <author>tc={6A98EA58-EBE2-D560-1FEC-96EE11A8B0CE}</author>
   </authors>
   <commentList>
     <comment ref="C4" authorId="0" xr:uid="{04CB6911-E216-5FFA-A00E-331AF1FB8FD4}">
@@ -59,12 +60,33 @@
         </r>
       </text>
     </comment>
+    <comment ref="D4" authorId="1" xr:uid="{6A98EA58-EBE2-D560-1FEC-96EE11A8B0CE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t>AskingMansOz:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">
+21.6 x Persona
+</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t xml:space="preserve">Integrantes Proyecto</t>
   </si>
@@ -81,7 +103,7 @@
     <t xml:space="preserve">Brandon Guido Navarro</t>
   </si>
   <si>
-    <t xml:space="preserve">Sebastián Obando</t>
+    <t xml:space="preserve">Sebastián Obando Ramírez</t>
   </si>
   <si>
     <t xml:space="preserve">Julián Solano Obando</t>
@@ -102,9 +124,6 @@
     <t xml:space="preserve">Historia de Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">Resumen Historia de Usuario (Justificación Story Points)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Story Points</t>
   </si>
   <si>
@@ -120,45 +139,30 @@
     <t xml:space="preserve">Servicio para Administrar Usuarios</t>
   </si>
   <si>
-    <t xml:space="preserve">Sube del CRUD estándar. Son 6 operaciones (una extra con filtros por identificación, nombre y tipo) y reglas de negocio propias: el dominio del email (cuc.cr o cuc.ac.cr) define qué rol es válido, el email es la llave única, la contraseña se guarda encriptada y los tipos de identificación deben poder extenderse. Se debe implementar token y bitácora.</t>
-  </si>
-  <si>
     <t>USR2</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Roles</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar. 5 operaciones sobre una entidad de 2 campos (identificador y nombre) con una sola validación (nombre solo letras y espacios), más token y bitácora.</t>
-  </si>
-  <si>
     <t>USR3</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Parametrización</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar. 5 operaciones sobre 2 campos (identificador y valor) con validaciones de formato (identificador de máximo 10 letras mayúsculas, valor de máximo 500 caracteres), más token y bitácora. Otras HU consumen sus valores, pero ese costo va en cada HU consumidora. Se debe implementar token y bitácora.</t>
-  </si>
-  <si>
     <t>USR4</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Módulos</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar. 5 operaciones sobre 2 campos (identificador y nombre), con validación de nombre solo letras y espacios, más token y bitácora.</t>
-  </si>
-  <si>
     <t>USR5</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Login</t>
   </si>
   <si>
-    <t xml:space="preserve">Login fijado en 5 por su complejidad base. 3 endpoints (/login, /refresh, /validate): /login verifica usuario y contraseña encriptada y responde 201 o 401, genera JWT y refresh token con expiración parametrizable; /refresh y /validate los consumen. Es crítico porque todas las demás HU validan su token contra /validate. Se debe implementar bitácora.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Oferta acádecima</t>
   </si>
   <si>
@@ -168,54 +172,36 @@
     <t xml:space="preserve">Servicio para Administrar Instituciones</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar. 5 operaciones sobre 2 campos (identificador y nombre de la institución), con validación de nombre solo letras y espacios, más token y bitácora.</t>
-  </si>
-  <si>
     <t>ACD2</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Carreras</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar de 4 campos (identificador, nombre, institución y director). Suma una consulta por institución y dos validaciones de existencia (la institución y que el director sea un profesor de ACD6), pero son lecturas, no lógica de negocio. Se debe implementar token y bitácora.</t>
-  </si>
-  <si>
     <t>ACD3</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Cursos</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar de 4 campos con una operación extra (cursos por carrera, 6 en total). Valida que la carrera exista y que el nivel esté entre 1 y 12. Se debe implementar token y bitácora.</t>
-  </si>
-  <si>
     <t>ACD4</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Grupos</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar de 7 campos con 3 relaciones (curso, profesor y periodo) más número, horario y cupo. Todo son validaciones de campo y de existencia; los criterios no piden reglas de negocio adicionales. Se debe implementar token y bitácora.</t>
-  </si>
-  <si>
     <t>ACD5</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Periodos</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar de 5 operaciones sobre 4 campos (año, número de periodo, fecha de inicio y fecha de fin); los criterios solo exigen que sean obligatorios, más token y bitácora.</t>
-  </si>
-  <si>
     <t>ACD6</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Profesores</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar de 6 campos. Suma validaciones de formato (nombre solo letras, mayor de edad, email del dominio parametrizable) y teléfonos múltiples, pero son validaciones de campo, no lógica de negocio. Se debe implementar token y bitácora. </t>
-  </si>
-  <si>
     <t>Matrícula</t>
   </si>
   <si>
@@ -225,45 +211,30 @@
     <t xml:space="preserve">Servicio para Administrar Pre-Matrícula</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar con encabezado (estudiante, carrera, periodo y observaciones opcionales) y lista de cursos. Las reglas (solo cursos de primer nivel y periodos futuros) son validaciones de lectura contra ACD3 y ACD5; no hay cálculos ni cambios de estado en otras entidades. Se debe implementar token y bitácora. </t>
-  </si>
-  <si>
     <t>MAT2</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Matrícula</t>
   </si>
   <si>
-    <t xml:space="preserve">Una operación menos que un CRUD (4: matricular, modificar, eliminar y consultar estudiantes por curso y grupo), pero contiene validaciones cruzadas: periodo activo y existencia de estudiante, curso y grupo. No calcula ni cambia estados en otras entidades. Se debe implementar token y bitácora. </t>
-  </si>
-  <si>
     <t>MAT3</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Expedientes de Estudiantes</t>
   </si>
   <si>
-    <t xml:space="preserve">CRUD estándar de 7 campos (identificación, tipo, email, nombre, fecha de nacimiento, dirección estructurada y teléfonos múltiples). Suma validaciones de formato (nombre solo letras, email con dominio parametrizable), sin lógica de negocio. Se debe implementar token y bitácora. </t>
-  </si>
-  <si>
     <t>MAT4</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Direcciones</t>
   </si>
   <si>
-    <t xml:space="preserve">Solo lectura. 3 consultas (/provincias, /cantones y /distritos) que no crean ni modifican datos. La única regla es que el cantón corresponda a la provincia; el trabajo extra es cargar el catálogo geográfico. Se debe implementar token y bitácora. </t>
-  </si>
-  <si>
     <t>MAT5</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Admininstrar Notas</t>
   </si>
   <si>
-    <t xml:space="preserve">Sube del CRUD por reglas de negocio con estado que controlar. 4 operaciones donde los rubros de un desglose deben sumar 100, cargar un desglose nuevo reemplaza el anterior, los rubros no se pueden modificar una vez asignadas notas y cada nota debe ir de 1 a 100. Se debe implementar token y bitácora. </t>
-  </si>
-  <si>
     <t>Académico</t>
   </si>
   <si>
@@ -273,18 +244,12 @@
     <t xml:space="preserve">Servicio para Consultar Historial Académico</t>
   </si>
   <si>
-    <t xml:space="preserve">Un solo endpoint de solo lectura (/historialacademico) que devuelve código, nombre y promedio por curso. No escribe ni cambia estados. Se debe implementar token y bitácora. </t>
-  </si>
-  <si>
     <t>ACA2</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Consultar Listado de Estudiantes</t>
   </si>
   <si>
-    <t xml:space="preserve">Un solo endpoint de solo lectura (/listadoestudiantes) que recibe un periodo y devuelve 7 datos por estudiante. Solo une información de otras entidades (estudiante, carrera, curso y grupo), sin cálculos.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Integración de pagos y notificaciones</t>
   </si>
   <si>
@@ -294,27 +259,18 @@
     <t xml:space="preserve">Servicio para Administrar Facturación</t>
   </si>
   <si>
-    <t xml:space="preserve">Sube del CRUD por lógica de negocio. 4 operaciones con patrón encabezado-detalle obligatorio, monto de 30.000 colones más impuesto del 2 %, detalle fijo "Servicios estudiantiles", estado inicial pendiente y anulación (reverso) de facturas. Se debe implementar token y bitácora.</t>
-  </si>
-  <si>
     <t>IPN2</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Administrar Pagos</t>
   </si>
   <si>
-    <t xml:space="preserve">Sube del CRUD por manejo de estados entre entidades. Crear un pago marca la factura como pagada y reversarlo la devuelve a pendiente, por lo que factura y pago deben mantenerse consistentes. 4 operaciones (crear, reversar, obtener uno y listar por periodo). Se debe implementar token y bitácora.</t>
-  </si>
-  <si>
     <t>IPN3</t>
   </si>
   <si>
     <t xml:space="preserve">Servicio para Gestiónar Notificaciones</t>
   </si>
   <si>
-    <t xml:space="preserve">Un solo endpoint (/notificar), pero con dependencia externa: envía correo con cuerpo HTML por un servidor de correo cuyos datos (servidor y cuenta) son parametrizables. Se debe implementar token y bitácora.</t>
-  </si>
-  <si>
     <t>General</t>
   </si>
   <si>
@@ -322,9 +278,6 @@
   </si>
   <si>
     <t xml:space="preserve">Servicio para Registrar y Consultar Bitácoras</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Técnicamente simple (2 endpoint /bitacora con 2 parámetros y fecha automática), pero es transversal: todos los demás servicios deben invocarlo para registrar cada operación de CRUD y cada error técnico. Además está implícito, se debe consultar el historial de bitácora.</t>
   </si>
 </sst>
 </file>
@@ -624,7 +577,7 @@
     <xf fontId="2" fillId="3" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0"/>
     <xf fontId="3" fillId="4" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="47">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -666,9 +619,6 @@
     <xf fontId="4" fillId="9" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="9" borderId="8" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="6" fillId="0" borderId="8" numFmtId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -681,9 +631,6 @@
     <xf fontId="4" fillId="9" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="9" borderId="10" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="6" fillId="0" borderId="10" numFmtId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -696,9 +643,6 @@
     <xf fontId="4" fillId="9" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="9" borderId="12" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="6" fillId="0" borderId="12" numFmtId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -711,9 +655,6 @@
     <xf fontId="4" fillId="10" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="10" borderId="8" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="6" fillId="0" borderId="8" numFmtId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -726,9 +667,6 @@
     <xf fontId="4" fillId="10" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="10" borderId="10" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="4" fillId="10" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -738,9 +676,6 @@
     <xf fontId="4" fillId="10" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="10" borderId="12" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="4" fillId="10" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -767,9 +702,6 @@
     </xf>
     <xf fontId="4" fillId="10" borderId="13" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="10" borderId="14" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="6" fillId="0" borderId="14" numFmtId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -805,7 +737,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="AskingMansOz" id="{CE720F10-A9C9-3E8C-67D9-3B74414113DB}" userId="AskingMansOz" providerId="Teamlab"/>
+  <person displayName="AskingMansOz" id="{A36F4E31-68DB-11C5-CF8D-E4A86219E6FC}" userId="AskingMansOz" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -1289,12 +1221,16 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C4" dT="2026-09-19T09:13:08.03Z" personId="{CE720F10-A9C9-3E8C-67D9-3B74414113DB}" id="{04CB6911-E216-5FFA-A00E-331AF1FB8FD4}" done="0">
+  <threadedComment ref="C4" dT="2026-09-19T09:13:08.03Z" personId="{A36F4E31-68DB-11C5-CF8D-E4A86219E6FC}" id="{04CB6911-E216-5FFA-A00E-331AF1FB8FD4}" done="0">
     <text xml:space="preserve">Mide la carga de trabajo del equipo con base en el promedio de puntos acumulados por los integrantes:
 * Verde: Por debajo del promedio (menor carga).
 * Amarillo: En el promedio exacto (carga equilibrada).
 * Rojo: Por encima del promedio (sobrecarga de trabajo).
 Lo ideal es que la carga de trabajo se mantengan cerca del promedio.
+</text>
+  </threadedComment>
+  <threadedComment ref="D4" dT="2026-09-25T19:25:05.93Z" personId="{A36F4E31-68DB-11C5-CF8D-E4A86219E6FC}" id="{6A98EA58-EBE2-D560-1FEC-96EE11A8B0CE}" done="0">
+    <text xml:space="preserve">21.6 x Persona
 </text>
   </threadedComment>
 </ThreadedComments>
@@ -1304,11 +1240,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.25"/>
   <cols>
-    <col bestFit="1" min="2" max="2" width="33"/>
+    <col customWidth="1" min="2" max="2" width="33.28125"/>
     <col customWidth="1" min="3" max="3" width="17.140625"/>
     <col customWidth="1" min="4" max="4" width="47.7109375"/>
-    <col customWidth="1" min="5" max="5" style="1" width="70.140625"/>
-    <col customWidth="1" min="6" max="6" width="12.140625"/>
+    <col bestFit="1" customWidth="1" min="5" max="5" style="1" width="11.34375"/>
+    <col customWidth="1" min="6" max="6" width="27.00390625"/>
     <col customWidth="1" min="7" max="7" width="18.421875"/>
     <col bestFit="1" customWidth="1" min="8" max="8" width="11.421875"/>
     <col bestFit="1" min="9" max="9" width="11.421875"/>
@@ -1337,12 +1273,12 @@
         <v>3</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" ref="C4:C8" si="0">SUMIF($G$13:$G$100,B4,$F$13:$F$100)</f>
-        <v>0</v>
+        <f t="shared" ref="C4:C8" si="0">SUMIF($F$13:$F$100,B4,$E$13:$E$100)</f>
+        <v>21</v>
       </c>
       <c r="D4" s="6">
-        <f t="shared" ref="D4:D8" si="1">COUNTIF($G$13:$G$100,B4)</f>
-        <v>0</v>
+        <f t="shared" ref="D4:D8" si="1">COUNTIF($E$13:$F$100,B4)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1351,11 +1287,11 @@
       </c>
       <c r="C5" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D5" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" ht="42.75">
@@ -1364,11 +1300,11 @@
       </c>
       <c r="C6" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D6" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" ht="28.5">
@@ -1377,11 +1313,11 @@
       </c>
       <c r="C7" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="D7" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" ht="28.5">
@@ -1390,11 +1326,11 @@
       </c>
       <c r="C8" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="D8" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H8" s="10"/>
     </row>
@@ -1404,7 +1340,7 @@
       </c>
       <c r="C9" s="12">
         <f>SUM(C4:C8)</f>
-        <v>0</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" ht="15"/>
@@ -1425,416 +1361,392 @@
       <c r="F12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>14</v>
-      </c>
     </row>
     <row r="13" ht="71.25">
       <c r="B13" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="D13" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="E13" s="15">
+        <v>8</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" ht="42.75">
+      <c r="B14" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="D14" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="16">
+      <c r="E14" s="19">
+        <v>5</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" ht="71.25">
+      <c r="B15" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="19">
+        <v>5</v>
+      </c>
+      <c r="F15" s="20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" ht="28.5">
+      <c r="B16" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="19">
+        <v>5</v>
+      </c>
+      <c r="F16" s="20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" ht="71.25">
+      <c r="B17" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="23">
         <v>8</v>
       </c>
-      <c r="G13" s="17"/>
-    </row>
-    <row r="14" ht="42.75">
-      <c r="B14" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="21">
-        <v>5</v>
-      </c>
-      <c r="G14" s="22"/>
-    </row>
-    <row r="15" ht="71.25">
-      <c r="B15" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E15" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="F15" s="21">
-        <v>5</v>
-      </c>
-      <c r="G15" s="22"/>
-    </row>
-    <row r="16" ht="28.5">
-      <c r="B16" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="19" t="s">
+      <c r="F17" s="24" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" ht="42.75">
+      <c r="B18" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="C18" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="20" t="s">
+      <c r="D18" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="21">
-        <v>5</v>
-      </c>
-      <c r="G16" s="22"/>
-    </row>
-    <row r="17" ht="71.25">
-      <c r="B17" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="24" t="s">
+      <c r="E18" s="27">
+        <v>5</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" ht="57">
+      <c r="B19" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D19" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="25" t="s">
+      <c r="E19" s="19">
+        <v>5</v>
+      </c>
+      <c r="F19" s="31" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" ht="42.75">
+      <c r="B20" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="F17" s="26">
-        <v>5</v>
-      </c>
-      <c r="G17" s="27"/>
-    </row>
-    <row r="18" ht="42.75">
-      <c r="B18" s="28" t="s">
+      <c r="D20" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="E20" s="19">
+        <v>5</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" ht="57">
+      <c r="B21" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D21" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="E18" s="30" t="s">
+      <c r="E21" s="19">
+        <v>5</v>
+      </c>
+      <c r="F21" s="31" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" ht="42.75">
+      <c r="B22" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="F18" s="31">
-        <v>5</v>
-      </c>
-      <c r="G18" s="32"/>
-    </row>
-    <row r="19" ht="57">
-      <c r="B19" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="34" t="s">
+      <c r="D22" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="33" t="s">
+      <c r="E22" s="19">
+        <v>5</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" ht="57">
+      <c r="B23" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="35" t="s">
+      <c r="D23" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="F19" s="21">
-        <v>5</v>
-      </c>
-      <c r="G19" s="36"/>
-    </row>
-    <row r="20" ht="42.75">
-      <c r="B20" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="D20" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="F20" s="21">
-        <v>5</v>
-      </c>
-      <c r="G20" s="36"/>
-    </row>
-    <row r="21" ht="57">
-      <c r="B21" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" s="33" t="s">
-        <v>42</v>
-      </c>
-      <c r="E21" s="35" t="s">
-        <v>43</v>
-      </c>
-      <c r="F21" s="21">
-        <v>5</v>
-      </c>
-      <c r="G21" s="36"/>
-    </row>
-    <row r="22" ht="42.75">
-      <c r="B22" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="33" t="s">
-        <v>45</v>
-      </c>
-      <c r="E22" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="F22" s="21">
-        <v>5</v>
-      </c>
-      <c r="G22" s="36"/>
-    </row>
-    <row r="23" ht="57">
-      <c r="B23" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="E23" s="39" t="s">
-        <v>49</v>
-      </c>
-      <c r="F23" s="26">
-        <v>5</v>
-      </c>
-      <c r="G23" s="40"/>
+      <c r="E23" s="23">
+        <v>5</v>
+      </c>
+      <c r="F23" s="34" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="24" ht="57">
       <c r="B24" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24" s="15">
+        <v>5</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" ht="57">
+      <c r="B25" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" s="35">
+        <v>5</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" ht="57">
+      <c r="B26" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="19">
+        <v>5</v>
+      </c>
+      <c r="F26" s="20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" ht="57">
+      <c r="B27" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" s="37">
+        <v>3</v>
+      </c>
+      <c r="F27" s="20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" ht="57">
+      <c r="B28" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="38">
+        <v>8</v>
+      </c>
+      <c r="F28" s="24" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" ht="42.75">
+      <c r="B29" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="D29" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="E29" s="39">
+        <v>3</v>
+      </c>
+      <c r="F29" s="28" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" ht="42.75">
+      <c r="B30" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="D30" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="F24" s="16">
-        <v>8</v>
-      </c>
-      <c r="G24" s="17"/>
-    </row>
-    <row r="25" ht="57">
-      <c r="B25" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D25" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="E25" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="F25" s="41">
-        <v>8</v>
-      </c>
-      <c r="G25" s="22"/>
-    </row>
-    <row r="26" ht="57">
-      <c r="B26" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D26" s="42" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="F26" s="21">
-        <v>5</v>
-      </c>
-      <c r="G26" s="22"/>
-    </row>
-    <row r="27" ht="57">
-      <c r="B27" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="F27" s="43">
+      <c r="E30" s="40">
         <v>3</v>
       </c>
-      <c r="G27" s="22"/>
-    </row>
-    <row r="28" ht="57">
-      <c r="B28" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="D28" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="E28" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="F28" s="44">
-        <v>8</v>
-      </c>
-      <c r="G28" s="27"/>
-    </row>
-    <row r="29" ht="42.75">
-      <c r="B29" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="C29" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="D29" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="E29" s="30" t="s">
-        <v>69</v>
-      </c>
-      <c r="F29" s="45">
-        <v>3</v>
-      </c>
-      <c r="G29" s="32"/>
-    </row>
-    <row r="30" ht="42.75">
-      <c r="B30" s="37" t="s">
-        <v>66</v>
-      </c>
-      <c r="C30" s="38" t="s">
-        <v>70</v>
-      </c>
-      <c r="D30" s="37" t="s">
-        <v>71</v>
-      </c>
-      <c r="E30" s="39" t="s">
-        <v>72</v>
-      </c>
-      <c r="F30" s="46">
-        <v>3</v>
-      </c>
-      <c r="G30" s="40"/>
+      <c r="F30" s="34" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="31" ht="57">
       <c r="B31" s="13" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="F31" s="16">
+        <v>56</v>
+      </c>
+      <c r="E31" s="15">
+        <v>5</v>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" ht="57">
+      <c r="B32" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="E32" s="35">
+        <v>5</v>
+      </c>
+      <c r="F32" s="20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" ht="42.75">
+      <c r="B33" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="E33" s="40">
+        <v>3</v>
+      </c>
+      <c r="F33" s="24" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" ht="57">
+      <c r="B34" s="41" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" s="42" t="s">
+        <v>62</v>
+      </c>
+      <c r="D34" s="41" t="s">
+        <v>63</v>
+      </c>
+      <c r="E34" s="43">
+        <v>2</v>
+      </c>
+      <c r="F34" s="44" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="D35" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="G31" s="17"/>
-    </row>
-    <row r="32" ht="57">
-      <c r="B32" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="C32" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="D32" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="E32" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="F32" s="41">
-        <v>8</v>
-      </c>
-      <c r="G32" s="22"/>
-    </row>
-    <row r="33" ht="42.75">
-      <c r="B33" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="C33" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="D33" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="E33" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="F33" s="46">
-        <v>3</v>
-      </c>
-      <c r="G33" s="27"/>
-    </row>
-    <row r="34" ht="57">
-      <c r="B34" s="47" t="s">
-        <v>83</v>
-      </c>
-      <c r="C34" s="48" t="s">
-        <v>84</v>
-      </c>
-      <c r="D34" s="47" t="s">
-        <v>85</v>
-      </c>
-      <c r="E34" s="49" t="s">
-        <v>86</v>
-      </c>
-      <c r="F34" s="50">
-        <v>5</v>
-      </c>
-      <c r="G34" s="51"/>
-    </row>
-    <row r="35" ht="14.25">
-      <c r="E35" s="52" t="s">
-        <v>8</v>
-      </c>
-      <c r="F35" s="53">
-        <f>SUM(F13:F34)</f>
-        <v>120</v>
+      <c r="E35" s="46">
+        <f>SUM(E13:E34)</f>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="O5mJHy0ukKPOr8Di3KTpE44BwJOcp+orMlh9xO42OUOfF1wcVZ6DnHIurUGeuQ3cg6s+xSnWbMilRkzzE52hTw==" saltValue="ZHjE9ECT6JLGntzd65jL9g==" spinCount="100000" autoFilter="1" deleteColumns="1" deleteRows="1" formatCells="1" formatColumns="1" formatRows="1" insertColumns="1" insertHyperlinks="1" insertRows="1" objects="0" pivotTables="1" scenarios="0" selectLockedCells="0" selectUnlockedCells="0" sheet="1" sort="1"/>
   <dataValidations count="1" disablePrompts="0">
     <dataValidation sqref="B4:B8" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1"/>
   </dataValidations>
@@ -1847,7 +1759,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{09BB8211-5B0D-45A9-8802-F9F642820BFB}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{A491789D-33FE-4324-BC33-CF6B8CB06D32}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -1855,10 +1767,10 @@
               </font>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F13:F34</xm:sqref>
+          <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="lessThanOrEqual" id="{A9EC28CA-90E4-44F3-8FE0-32656C7F0A1A}">
+          <x14:cfRule type="cellIs" priority="7" operator="lessThanOrEqual" id="{621659AE-3BB9-4F31-B6FD-E7E5C443857F}">
             <xm:f>3</xm:f>
             <x14:dxf>
               <font>
@@ -1872,10 +1784,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F13:F34</xm:sqref>
+          <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="notBetween" id="{3B2FCBEF-CCE7-4E53-8C5D-2B0883AC9268}">
+          <x14:cfRule type="cellIs" priority="6" operator="notBetween" id="{1CB83144-0E53-49D1-ACD6-5E9B38DCFEAA}">
             <xm:f>3</xm:f>
             <xm:f>8</xm:f>
             <x14:dxf>
@@ -1890,10 +1802,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F13:F34</xm:sqref>
+          <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="between" id="{DEF280EA-0099-4633-BBF2-379C4AB18D4D}">
+          <x14:cfRule type="cellIs" priority="5" operator="between" id="{D9ECC498-759E-4113-AF0C-6FF6F5A0B5FA}">
             <xm:f>4</xm:f>
             <xm:f>7</xm:f>
             <x14:dxf>
@@ -1908,10 +1820,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F13:F34</xm:sqref>
+          <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" id="{F4608307-6605-4A03-8D0F-504D7B2BDC85}">
+          <x14:cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" id="{C9C416E8-F46A-469F-B328-5E5348235630}">
             <xm:f>8</xm:f>
             <x14:dxf>
               <font>
@@ -1925,10 +1837,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F13:F34</xm:sqref>
+          <xm:sqref>E13:E34</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="aboveAverage" priority="2" stdDev="0" id="{56553315-77DA-4C89-9131-296A3670719A}">
+          <x14:cfRule type="aboveAverage" priority="3" stdDev="0" id="{DBCBFC1D-BC2D-4E42-92C6-5A4FA61E3E8D}">
             <x14:dxf>
               <font>
                 <color rgb="FF9C0006"/>
@@ -1944,7 +1856,7 @@
           <xm:sqref>C4:C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="aboveAverage" priority="1" aboveAverage="0" stdDev="0" id="{E7FA339C-0920-4A26-A157-52581599B7CF}">
+          <x14:cfRule type="aboveAverage" priority="2" aboveAverage="0" stdDev="0" id="{755BB3AC-D42C-4BD3-88DC-81419C3E7F68}">
             <x14:dxf>
               <font>
                 <color rgb="FF006100"/>
@@ -1959,15 +1871,32 @@
           </x14:cfRule>
           <xm:sqref>C4:C8</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="1" operator="lessThan" id="{543E6632-DA0C-419B-B3DA-03DDB1AE2DED}">
+            <xm:f>5</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E34</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{C71EC464-344C-4E81-9097-7A8AE933C8F4}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{22371375-5570-4B72-8497-72B6EB5465DB}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>
-          <xm:sqref>G13:G34</xm:sqref>
+          <xm:sqref>F13:F34</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>